<commit_message>
data: live v2.1 market ranking refresh
</commit_message>
<xml_diff>
--- a/reports/investment_dashboard.xlsx
+++ b/reports/investment_dashboard.xlsx
@@ -1091,7 +1091,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>44.96</v>
+        <v>44.95</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1478,16 +1478,16 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MongoDB, Inc.</t>
+          <t>Palo Alto Networks, Inc.</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>42.18</v>
+        <v>42.21</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1495,11 +1495,11 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>362.2099914550781</v>
+        <v>330.6499938964844</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="H21" t="n">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Revenue Growth; Balance Sheet</t>
+          <t>Revenue Growth</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Very high earnings multiple</t>
+          <t>Excessive price-to-sales valuation; Very high earnings multiple</t>
         </is>
       </c>
     </row>
@@ -1530,16 +1530,16 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Palo Alto Networks, Inc.</t>
+          <t>MongoDB, Inc.</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>42.13</v>
+        <v>42.17</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1547,11 +1547,11 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>330.6499938964844</v>
+        <v>362.2099914550781</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="H22" t="n">
@@ -1562,7 +1562,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Revenue Growth</t>
+          <t>Revenue Growth; Balance Sheet</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1572,7 +1572,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Excessive price-to-sales valuation; Very high earnings multiple</t>
+          <t>Very high earnings multiple</t>
         </is>
       </c>
     </row>
@@ -1931,16 +1931,16 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ServiceNow, Inc.</t>
+          <t>Oracle Corporation</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>35.18</v>
+        <v>36.39</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1948,22 +1948,32 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>132.5299987792969</v>
+        <v>150.2799987792969</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="H30" t="n">
-        <v>100</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="I30" t="n">
-        <v>100</v>
+        <v>94.09999999999999</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Revenue Growth</t>
+        </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Earnings Fcf; Industry Growth; Valuation; Competitive Advantage; Catalysts; Inflation Resilience</t>
+          <t>Industry Growth; Balance Sheet; Competitive Advantage; Momentum; Catalysts; Inflation Resilience</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Negative free cash flow / unprofitable growth; Debt materially exceeds cash</t>
         </is>
       </c>
     </row>
@@ -1973,16 +1983,16 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Oracle Corporation</t>
+          <t>ServiceNow, Inc.</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>30.22</v>
+        <v>35.18</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1990,27 +2000,22 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>150.2799987792969</v>
+        <v>132.5299987792969</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="H31" t="n">
-        <v>94.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="I31" t="n">
-        <v>94.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Industry Growth; Balance Sheet; Competitive Advantage; Momentum; Catalysts; Inflation Resilience</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>Negative free cash flow / unprofitable growth; Debt materially exceeds cash</t>
+          <t>Earnings Fcf; Industry Growth; Valuation; Competitive Advantage; Catalysts; Inflation Resilience</t>
         </is>
       </c>
     </row>
@@ -2585,7 +2590,7 @@
         <v>2.55</v>
       </c>
       <c r="I13" t="n">
-        <v>3.53</v>
+        <v>3.52</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -2594,7 +2599,7 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>44.96</v>
+        <v>44.95</v>
       </c>
     </row>
     <row r="14">
@@ -2880,32 +2885,32 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>13.31</v>
+        <v>14.81</v>
       </c>
       <c r="C21" t="n">
-        <v>8.42</v>
+        <v>8.85</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>9.890000000000001</v>
+        <v>7.72</v>
       </c>
       <c r="F21" t="n">
-        <v>2.33</v>
+        <v>0.73</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>4.49</v>
+        <v>6.53</v>
       </c>
       <c r="I21" t="n">
-        <v>3.74</v>
+        <v>3.57</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -2914,38 +2919,38 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>42.18</v>
+        <v>42.21</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>14.78</v>
+        <v>13.31</v>
       </c>
       <c r="C22" t="n">
-        <v>8.76</v>
+        <v>8.42</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>7.76</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="F22" t="n">
-        <v>0.73</v>
+        <v>2.32</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>6.53</v>
+        <v>4.49</v>
       </c>
       <c r="I22" t="n">
-        <v>3.57</v>
+        <v>3.74</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -2954,7 +2959,7 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>42.13</v>
+        <v>42.17</v>
       </c>
     </row>
     <row r="23">
@@ -3240,32 +3245,32 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>10.88</v>
+        <v>12.97</v>
       </c>
       <c r="C30" t="n">
-        <v>5.68</v>
+        <v>10</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
       </c>
       <c r="E30" t="n">
-        <v>6.78</v>
+        <v>0.9</v>
       </c>
       <c r="F30" t="n">
-        <v>3.85</v>
+        <v>7.78</v>
       </c>
       <c r="G30" t="n">
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>4.43</v>
+        <v>1.16</v>
       </c>
       <c r="I30" t="n">
-        <v>3.56</v>
+        <v>3.58</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -3274,38 +3279,38 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>35.18</v>
+        <v>36.39</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>9.6</v>
+        <v>10.88</v>
       </c>
       <c r="C31" t="n">
-        <v>8.539999999999999</v>
+        <v>5.68</v>
       </c>
       <c r="D31" t="n">
         <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>0.8</v>
+        <v>6.78</v>
       </c>
       <c r="F31" t="n">
-        <v>6.54</v>
+        <v>3.85</v>
       </c>
       <c r="G31" t="n">
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>1.16</v>
+        <v>4.43</v>
       </c>
       <c r="I31" t="n">
-        <v>3.58</v>
+        <v>3.56</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -3314,7 +3319,7 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>30.22</v>
+        <v>35.18</v>
       </c>
     </row>
   </sheetData>
@@ -3353,7 +3358,7 @@
     <col width="19" customWidth="1" min="19" max="19"/>
     <col width="23" customWidth="1" min="20" max="20"/>
     <col width="23" customWidth="1" min="21" max="21"/>
-    <col width="23" customWidth="1" min="22" max="22"/>
+    <col width="22" customWidth="1" min="22" max="22"/>
     <col width="23" customWidth="1" min="23" max="23"/>
     <col width="18" customWidth="1" min="24" max="24"/>
     <col width="24" customWidth="1" min="25" max="25"/>
@@ -3550,7 +3555,7 @@
         <v>0.36</v>
       </c>
       <c r="I2" t="n">
-        <v>13.57</v>
+        <v>13.56</v>
       </c>
       <c r="J2" t="n">
         <v>0.774</v>
@@ -3571,7 +3576,7 @@
         <v>0.60344005</v>
       </c>
       <c r="Q2" t="n">
-        <v>31.926308</v>
+        <v>31.94985</v>
       </c>
       <c r="R2" t="n">
         <v>0.5060223</v>
@@ -3589,17 +3594,17 @@
         <v>0.2872165910885389</v>
       </c>
       <c r="W2" t="n">
-        <v>0.6918288184435979</v>
+        <v>0.6918286168232719</v>
       </c>
       <c r="X2" t="n">
         <v>0.00013</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.15487</v>
+        <v>0.1549</v>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>2026-09-11T22:52:02.073420+00:00</t>
+          <t>2026-09-14T13:18:40.075592+00:00</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
@@ -3681,17 +3686,17 @@
         <v>1.289957921719005</v>
       </c>
       <c r="W3" t="n">
-        <v>5.487515560380774</v>
+        <v>5.4875162188819</v>
       </c>
       <c r="X3" t="n">
         <v>0.00238</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.79882</v>
+        <v>0.7988</v>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>2026-09-11T22:51:57.285743+00:00</t>
+          <t>2026-09-14T13:18:35.348604+00:00</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
@@ -3734,7 +3739,7 @@
         <v>0.577</v>
       </c>
       <c r="I4" t="n">
-        <v>17.17</v>
+        <v>17.19</v>
       </c>
       <c r="J4" t="n">
         <v>2.729</v>
@@ -3755,7 +3760,7 @@
         <v>0.12020001</v>
       </c>
       <c r="Q4" t="n">
-        <v>33.039604</v>
+        <v>33.00116</v>
       </c>
       <c r="R4" t="n">
         <v>2.3855643</v>
@@ -3770,20 +3775,20 @@
         <v>0.4364774763315671</v>
       </c>
       <c r="V4" t="n">
-        <v>2.759303711231271</v>
+        <v>2.759303331103376</v>
       </c>
       <c r="W4" t="n">
-        <v>3.582586931511815</v>
+        <v>3.582587213938946</v>
       </c>
       <c r="X4" t="n">
         <v>0.07719999600000001</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.77880996</v>
+        <v>0.77892995</v>
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>2026-09-11T22:52:04.504366+00:00</t>
+          <t>2026-09-14T13:18:42.316572+00:00</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
@@ -3826,7 +3831,7 @@
         <v>0.377</v>
       </c>
       <c r="I5" t="n">
-        <v>3.16</v>
+        <v>3.15</v>
       </c>
       <c r="J5" t="n">
         <v>0.357</v>
@@ -3847,7 +3852,7 @@
         <v>0.45393002</v>
       </c>
       <c r="Q5" t="n">
-        <v>63.16139</v>
+        <v>63.3619</v>
       </c>
       <c r="R5" t="n">
         <v>23.881285</v>
@@ -3871,11 +3876,11 @@
         <v>0.17247</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.73320997</v>
+        <v>0.73328</v>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>2026-09-11T22:52:03.831802+00:00</t>
+          <t>2026-09-14T13:18:41.869638+00:00</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
@@ -3957,17 +3962,17 @@
         <v>0.3267553938009435</v>
       </c>
       <c r="W6" t="n">
-        <v>2.292276885215299</v>
+        <v>2.292276667434656</v>
       </c>
       <c r="X6" t="n">
         <v>0.00202</v>
       </c>
       <c r="Y6" t="n">
-        <v>1.0058999</v>
+        <v>1.00614</v>
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>2026-09-11T22:51:58.401956+00:00</t>
+          <t>2026-09-14T13:18:36.491262+00:00</t>
         </is>
       </c>
       <c r="AD6" t="inlineStr">
@@ -4046,7 +4051,7 @@
         <v>0.06503360332428509</v>
       </c>
       <c r="V7" t="n">
-        <v>0.2138082500949225</v>
+        <v>0.2138083530828809</v>
       </c>
       <c r="W7" t="n">
         <v>0.2350453814344682</v>
@@ -4055,11 +4060,11 @@
         <v>0.04007</v>
       </c>
       <c r="Y7" t="n">
-        <v>0.71406</v>
+        <v>0.71410006</v>
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>2026-09-11T22:51:55.259473+00:00</t>
+          <t>2026-09-14T13:18:33.241504+00:00</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
@@ -4102,7 +4107,7 @@
         <v>0.928</v>
       </c>
       <c r="I8" t="n">
-        <v>1.18</v>
+        <v>1.17</v>
       </c>
       <c r="J8" t="n">
         <v>2.154</v>
@@ -4123,7 +4128,7 @@
         <v>0.47120997</v>
       </c>
       <c r="Q8" t="n">
-        <v>141.72034</v>
+        <v>142.93163</v>
       </c>
       <c r="R8" t="n">
         <v>65.28059</v>
@@ -4147,11 +4152,11 @@
         <v>0.03477</v>
       </c>
       <c r="Y8" t="n">
-        <v>0.6477300499999999</v>
+        <v>0.64741</v>
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>2026-09-11T22:51:55.589771+00:00</t>
+          <t>2026-09-14T13:18:33.607751+00:00</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr">
@@ -4239,11 +4244,11 @@
         <v>0.09433</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.73612</v>
+        <v>0.73567003</v>
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>2026-09-11T22:51:57.907207+00:00</t>
+          <t>2026-09-14T13:18:36.099860+00:00</t>
         </is>
       </c>
       <c r="AD9" t="inlineStr">
@@ -4286,7 +4291,7 @@
         <v>0.501</v>
       </c>
       <c r="I10" t="n">
-        <v>3.93</v>
+        <v>3.92</v>
       </c>
       <c r="J10" t="n">
         <v>1.595</v>
@@ -4307,7 +4312,7 @@
         <v>0.1725</v>
       </c>
       <c r="Q10" t="n">
-        <v>131.3308</v>
+        <v>131.66582</v>
       </c>
       <c r="R10" t="n">
         <v>20.398724</v>
@@ -4331,11 +4336,11 @@
         <v>0.00424</v>
       </c>
       <c r="Y10" t="n">
-        <v>0.75388</v>
+        <v>0.75382006</v>
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>2026-09-11T22:51:56.005502+00:00</t>
+          <t>2026-09-14T13:18:33.971595+00:00</t>
         </is>
       </c>
       <c r="AD10" t="inlineStr">
@@ -4378,7 +4383,7 @@
         <v>0.242</v>
       </c>
       <c r="I11" t="n">
-        <v>19.92</v>
+        <v>19.94</v>
       </c>
       <c r="J11" t="n">
         <v>2.94</v>
@@ -4399,7 +4404,7 @@
         <v>0.34033</v>
       </c>
       <c r="Q11" t="n">
-        <v>16.992971</v>
+        <v>16.975927</v>
       </c>
       <c r="R11" t="n">
         <v>9.284927</v>
@@ -4417,17 +4422,17 @@
         <v>0.1212118179624675</v>
       </c>
       <c r="W11" t="n">
-        <v>0.4119080505594885</v>
+        <v>0.4119079606978782</v>
       </c>
       <c r="X11" t="n">
         <v>0.01596</v>
       </c>
       <c r="Y11" t="n">
-        <v>0.80988</v>
+        <v>0.81016</v>
       </c>
       <c r="AC11" t="inlineStr">
         <is>
-          <t>2026-09-11T22:52:00.171768+00:00</t>
+          <t>2026-09-14T13:18:38.376538+00:00</t>
         </is>
       </c>
       <c r="AD11" t="inlineStr">
@@ -4506,7 +4511,7 @@
         <v>-0.1556730262276915</v>
       </c>
       <c r="V12" t="n">
-        <v>1.689238258735586</v>
+        <v>1.689238025038875</v>
       </c>
       <c r="W12" t="n">
         <v>2.553132104648163</v>
@@ -4515,11 +4520,11 @@
         <v>0.00494</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.81848997</v>
+        <v>0.81794</v>
       </c>
       <c r="AC12" t="inlineStr">
         <is>
-          <t>2026-09-11T22:52:03.441932+00:00</t>
+          <t>2026-09-14T13:18:41.501487+00:00</t>
         </is>
       </c>
       <c r="AD12" t="inlineStr">
@@ -4568,7 +4573,7 @@
         <v>2.153</v>
       </c>
       <c r="K13" t="n">
-        <v>30497124352</v>
+        <v>30596499456</v>
       </c>
       <c r="M13" t="n">
         <v>23975000064</v>
@@ -4589,7 +4594,7 @@
         <v>19.39314</v>
       </c>
       <c r="S13" t="n">
-        <v>56.66128728332635</v>
+        <v>56.47725573015303</v>
       </c>
       <c r="T13" t="n">
         <v>-0.1299363036767943</v>
@@ -4601,17 +4606,17 @@
         <v>0.1277732642630893</v>
       </c>
       <c r="W13" t="n">
-        <v>0.01393734656336121</v>
+        <v>0.01393743323475483</v>
       </c>
       <c r="X13" t="n">
-        <v>0.01948</v>
+        <v>0.01941</v>
       </c>
       <c r="Y13" t="n">
-        <v>0.80167997</v>
+        <v>0.7982</v>
       </c>
       <c r="AC13" t="inlineStr">
         <is>
-          <t>2026-09-11T22:51:56.510237+00:00</t>
+          <t>2026-09-14T13:18:34.381653+00:00</t>
         </is>
       </c>
       <c r="AD13" t="inlineStr">
@@ -4699,11 +4704,11 @@
         <v>0.10837</v>
       </c>
       <c r="Y14" t="n">
-        <v>0.90419</v>
+        <v>0.90404</v>
       </c>
       <c r="AC14" t="inlineStr">
         <is>
-          <t>2026-09-11T22:52:08.727709+00:00</t>
+          <t>2026-09-14T13:18:45.588269+00:00</t>
         </is>
       </c>
       <c r="AD14" t="inlineStr">
@@ -4746,7 +4751,7 @@
         <v>0.248</v>
       </c>
       <c r="I15" t="n">
-        <v>11.58</v>
+        <v>11.59</v>
       </c>
       <c r="J15" t="n">
         <v>0.428</v>
@@ -4767,7 +4772,7 @@
         <v>0.33736</v>
       </c>
       <c r="Q15" t="n">
-        <v>39.42055</v>
+        <v>39.38654</v>
       </c>
       <c r="R15" t="n">
         <v>11.747877</v>
@@ -4791,11 +4796,11 @@
         <v>0.0033000002</v>
       </c>
       <c r="Y15" t="n">
-        <v>0.86241996</v>
+        <v>0.86244005</v>
       </c>
       <c r="AC15" t="inlineStr">
         <is>
-          <t>2026-09-11T22:51:56.871728+00:00</t>
+          <t>2026-09-14T13:18:34.896594+00:00</t>
         </is>
       </c>
       <c r="AD15" t="inlineStr">
@@ -4883,11 +4888,11 @@
         <v>0.00583</v>
       </c>
       <c r="Y16" t="n">
-        <v>0.92816</v>
+        <v>0.9281700000000001</v>
       </c>
       <c r="AC16" t="inlineStr">
         <is>
-          <t>2026-09-11T22:52:06.354693+00:00</t>
+          <t>2026-09-14T13:18:43.953012+00:00</t>
         </is>
       </c>
       <c r="AD16" t="inlineStr">
@@ -4918,7 +4923,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>26344310784</v>
+        <v>25939607552</v>
       </c>
       <c r="F17" t="n">
         <v>40.09999847412109</v>
@@ -4954,7 +4959,7 @@
         <v>12.300613</v>
       </c>
       <c r="R17" t="n">
-        <v>0.67440444</v>
+        <v>0.6640442</v>
       </c>
       <c r="T17" t="n">
         <v>0.06620573845681355</v>
@@ -4972,11 +4977,11 @@
         <v>0.12696</v>
       </c>
       <c r="Y17" t="n">
-        <v>0.69428</v>
+        <v>0.69434</v>
       </c>
       <c r="AC17" t="inlineStr">
         <is>
-          <t>2026-09-11T22:52:05.626042+00:00</t>
+          <t>2026-09-14T13:18:43.089325+00:00</t>
         </is>
       </c>
       <c r="AD17" t="inlineStr">
@@ -5061,11 +5066,11 @@
         <v>0.12675999</v>
       </c>
       <c r="Y18" t="n">
-        <v>0.77855</v>
+        <v>0.77859</v>
       </c>
       <c r="AC18" t="inlineStr">
         <is>
-          <t>2026-09-11T22:51:57.594575+00:00</t>
+          <t>2026-09-14T13:18:35.734092+00:00</t>
         </is>
       </c>
       <c r="AD18" t="inlineStr">
@@ -5108,7 +5113,7 @@
         <v>0.196</v>
       </c>
       <c r="I19" t="n">
-        <v>12.42</v>
+        <v>12.43</v>
       </c>
       <c r="J19" t="n">
         <v>2.423</v>
@@ -5129,7 +5134,7 @@
         <v>0.13689</v>
       </c>
       <c r="Q19" t="n">
-        <v>20.674719</v>
+        <v>20.658085</v>
       </c>
       <c r="R19" t="n">
         <v>3.5706854</v>
@@ -5157,7 +5162,7 @@
       </c>
       <c r="AC19" t="inlineStr">
         <is>
-          <t>2026-09-11T22:52:00.719343+00:00</t>
+          <t>2026-09-14T13:18:38.801739+00:00</t>
         </is>
       </c>
       <c r="AD19" t="inlineStr">
@@ -5200,7 +5205,7 @@
         <v>0.351</v>
       </c>
       <c r="I20" t="n">
-        <v>-3.17</v>
+        <v>-3.16</v>
       </c>
       <c r="K20" t="n">
         <v>1739526656</v>
@@ -5236,14 +5241,14 @@
         <v>0.4652384626686688</v>
       </c>
       <c r="X20" t="n">
-        <v>0.029059999</v>
+        <v>0.029000001</v>
       </c>
       <c r="Y20" t="n">
-        <v>0.8097299999999999</v>
+        <v>0.81003</v>
       </c>
       <c r="AC20" t="inlineStr">
         <is>
-          <t>2026-09-11T22:52:06.041195+00:00</t>
+          <t>2026-09-14T13:18:43.454562+00:00</t>
         </is>
       </c>
       <c r="AD20" t="inlineStr">
@@ -5255,12 +5260,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>MongoDB, Inc.</t>
+          <t>Palo Alto Networks, Inc.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -5274,65 +5279,65 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>29133248512</v>
+        <v>270471692288</v>
       </c>
       <c r="F21" t="n">
-        <v>362.2099914550781</v>
+        <v>330.6499938964844</v>
       </c>
       <c r="G21" t="n">
-        <v>2782769920</v>
+        <v>11480000512</v>
       </c>
       <c r="H21" t="n">
-        <v>0.305</v>
+        <v>0.345</v>
       </c>
       <c r="I21" t="n">
-        <v>0.71</v>
+        <v>0.4</v>
       </c>
       <c r="K21" t="n">
-        <v>561356224</v>
+        <v>4240624896</v>
       </c>
       <c r="M21" t="n">
-        <v>2411254016</v>
+        <v>3071000064</v>
       </c>
       <c r="N21" t="n">
-        <v>55013000</v>
+        <v>2567000064</v>
       </c>
       <c r="O21" t="n">
-        <v>0.72688</v>
+        <v>0.70383</v>
       </c>
       <c r="P21" t="n">
-        <v>0.0368</v>
+        <v>0.05396</v>
       </c>
       <c r="Q21" t="n">
-        <v>510.15494</v>
+        <v>826.625</v>
       </c>
       <c r="R21" t="n">
-        <v>10.469154</v>
+        <v>23.560251</v>
       </c>
       <c r="S21" t="n">
-        <v>51.89797007042715</v>
+        <v>63.78109333441031</v>
       </c>
       <c r="T21" t="n">
-        <v>-0.1727154316432506</v>
+        <v>-0.1456293492338157</v>
       </c>
       <c r="U21" t="n">
-        <v>0.05662194968872614</v>
+        <v>0.1824976742378901</v>
       </c>
       <c r="V21" t="n">
-        <v>0.3904414259312021</v>
+        <v>0.9797029423918147</v>
       </c>
       <c r="W21" t="n">
-        <v>0.09066541643536508</v>
+        <v>0.6671708306549862</v>
       </c>
       <c r="X21" t="n">
-        <v>0.02637</v>
+        <v>0.0075700004</v>
       </c>
       <c r="Y21" t="n">
-        <v>0.96744</v>
+        <v>0.84473</v>
       </c>
       <c r="AC21" t="inlineStr">
         <is>
-          <t>2026-09-11T22:52:08.403675+00:00</t>
+          <t>2026-09-14T13:18:37.504630+00:00</t>
         </is>
       </c>
       <c r="AD21" t="inlineStr">
@@ -5344,12 +5349,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Palo Alto Networks, Inc.</t>
+          <t>MongoDB, Inc.</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -5363,65 +5368,65 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>269479739392</v>
+        <v>29178312704</v>
       </c>
       <c r="F22" t="n">
-        <v>330.6499938964844</v>
+        <v>362.2099914550781</v>
       </c>
       <c r="G22" t="n">
-        <v>11480000512</v>
+        <v>2782769920</v>
       </c>
       <c r="H22" t="n">
-        <v>0.344</v>
+        <v>0.305</v>
       </c>
       <c r="I22" t="n">
-        <v>1.15</v>
+        <v>0.72</v>
       </c>
       <c r="K22" t="n">
-        <v>4469550080</v>
+        <v>561356224</v>
       </c>
       <c r="M22" t="n">
-        <v>3071000064</v>
+        <v>2411254016</v>
       </c>
       <c r="N22" t="n">
-        <v>2500000000</v>
+        <v>55013000</v>
       </c>
       <c r="O22" t="n">
-        <v>0.70488</v>
+        <v>0.72688</v>
       </c>
       <c r="P22" t="n">
-        <v>0.050440002</v>
+        <v>0.0368</v>
       </c>
       <c r="Q22" t="n">
-        <v>287.52173</v>
+        <v>503.06943</v>
       </c>
       <c r="R22" t="n">
-        <v>23.473845</v>
+        <v>10.485349</v>
       </c>
       <c r="S22" t="n">
-        <v>60.29236378799004</v>
+        <v>51.97824742386752</v>
       </c>
       <c r="T22" t="n">
-        <v>-0.1456293492338157</v>
+        <v>-0.1727154316432506</v>
       </c>
       <c r="U22" t="n">
-        <v>0.1824976742378901</v>
+        <v>0.05662194968872614</v>
       </c>
       <c r="V22" t="n">
-        <v>0.9797029423918147</v>
+        <v>0.3904414259312021</v>
       </c>
       <c r="W22" t="n">
-        <v>0.6671708306549862</v>
+        <v>0.09066541643536508</v>
       </c>
       <c r="X22" t="n">
-        <v>0.0075700004</v>
+        <v>0.02637</v>
       </c>
       <c r="Y22" t="n">
-        <v>0.84471</v>
+        <v>0.96753</v>
       </c>
       <c r="AC22" t="inlineStr">
         <is>
-          <t>2026-09-11T22:51:59.392563+00:00</t>
+          <t>2026-09-14T13:18:45.161872+00:00</t>
         </is>
       </c>
       <c r="AD22" t="inlineStr">
@@ -5464,7 +5469,7 @@
         <v>0.359</v>
       </c>
       <c r="I23" t="n">
-        <v>-0.59</v>
+        <v>-0.58</v>
       </c>
       <c r="K23" t="n">
         <v>691946368</v>
@@ -5507,7 +5512,7 @@
       </c>
       <c r="AC23" t="inlineStr">
         <is>
-          <t>2026-09-11T22:52:07.617027+00:00</t>
+          <t>2026-09-14T13:18:44.391089+00:00</t>
         </is>
       </c>
       <c r="AD23" t="inlineStr">
@@ -5586,7 +5591,7 @@
         <v>-0.1510764554471811</v>
       </c>
       <c r="V24" t="n">
-        <v>-0.006587415460754698</v>
+        <v>-0.00658729830195004</v>
       </c>
       <c r="W24" t="n">
         <v>0.8962725001561778</v>
@@ -5595,11 +5600,11 @@
         <v>0.00238</v>
       </c>
       <c r="Y24" t="n">
-        <v>0.84543</v>
+        <v>0.84540004</v>
       </c>
       <c r="AC24" t="inlineStr">
         <is>
-          <t>2026-09-11T22:52:05.133552+00:00</t>
+          <t>2026-09-14T13:18:42.723495+00:00</t>
         </is>
       </c>
       <c r="AD24" t="inlineStr">
@@ -5642,7 +5647,7 @@
         <v>0.28</v>
       </c>
       <c r="I25" t="n">
-        <v>26.55</v>
+        <v>26.57</v>
       </c>
       <c r="J25" t="n">
         <v>-0.134</v>
@@ -5663,7 +5668,7 @@
         <v>0.34827</v>
       </c>
       <c r="Q25" t="n">
-        <v>24.407911</v>
+        <v>24.389538</v>
       </c>
       <c r="R25" t="n">
         <v>7.232781</v>
@@ -5681,17 +5686,17 @@
         <v>0.05780582477842255</v>
       </c>
       <c r="W25" t="n">
-        <v>-0.1341670638786125</v>
+        <v>-0.1341671344864807</v>
       </c>
       <c r="X25" t="n">
         <v>0.00148</v>
       </c>
       <c r="Y25" t="n">
-        <v>0.79014</v>
+        <v>0.7902</v>
       </c>
       <c r="AC25" t="inlineStr">
         <is>
-          <t>2026-09-11T22:52:01.045258+00:00</t>
+          <t>2026-09-14T13:18:39.201356+00:00</t>
         </is>
       </c>
       <c r="AD25" t="inlineStr">
@@ -5734,7 +5739,7 @@
         <v>0.177</v>
       </c>
       <c r="I26" t="n">
-        <v>17.97</v>
+        <v>17.94</v>
       </c>
       <c r="J26" t="n">
         <v>0.317</v>
@@ -5755,7 +5760,7 @@
         <v>0.45111</v>
       </c>
       <c r="Q26" t="n">
-        <v>27.580969</v>
+        <v>27.62709</v>
       </c>
       <c r="R26" t="n">
         <v>11.090689</v>
@@ -5773,17 +5778,17 @@
         <v>0.258092683375748</v>
       </c>
       <c r="W26" t="n">
-        <v>-0.002599071124246732</v>
+        <v>-0.002599009870587476</v>
       </c>
       <c r="X26" t="n">
         <v>0.00091</v>
       </c>
       <c r="Y26" t="n">
-        <v>0.75791</v>
+        <v>0.75792</v>
       </c>
       <c r="AC26" t="inlineStr">
         <is>
-          <t>2026-09-11T22:51:59.740314+00:00</t>
+          <t>2026-09-14T13:18:37.972548+00:00</t>
         </is>
       </c>
       <c r="AD26" t="inlineStr">
@@ -5826,7 +5831,7 @@
         <v>0.213</v>
       </c>
       <c r="I27" t="n">
-        <v>29.53</v>
+        <v>29.55</v>
       </c>
       <c r="J27" t="n">
         <v>0.285</v>
@@ -5847,7 +5852,7 @@
         <v>0.37057</v>
       </c>
       <c r="Q27" t="n">
-        <v>57.511005</v>
+        <v>57.472084</v>
       </c>
       <c r="R27" t="n">
         <v>18.464851</v>
@@ -5865,17 +5870,17 @@
         <v>0.2664215470752866</v>
       </c>
       <c r="W27" t="n">
-        <v>1.125803490281717</v>
+        <v>1.125803652691395</v>
       </c>
       <c r="X27" t="n">
         <v>0.00016000001</v>
       </c>
       <c r="Y27" t="n">
-        <v>0.20393999</v>
+        <v>0.20397</v>
       </c>
       <c r="AC27" t="inlineStr">
         <is>
-          <t>2026-09-11T22:52:02.528390+00:00</t>
+          <t>2026-09-14T13:18:40.748418+00:00</t>
         </is>
       </c>
       <c r="AD27" t="inlineStr">
@@ -5918,7 +5923,7 @@
         <v>0.224</v>
       </c>
       <c r="I28" t="n">
-        <v>0.99</v>
+        <v>0.98</v>
       </c>
       <c r="J28" t="n">
         <v>1.083</v>
@@ -5939,7 +5944,7 @@
         <v>0.07603</v>
       </c>
       <c r="Q28" t="n">
-        <v>267.46466</v>
+        <v>270.19388</v>
       </c>
       <c r="R28" t="n">
         <v>54.84782</v>
@@ -5967,7 +5972,7 @@
       </c>
       <c r="AC28" t="inlineStr">
         <is>
-          <t>2026-09-11T22:52:03.056920+00:00</t>
+          <t>2026-09-14T13:18:41.110406+00:00</t>
         </is>
       </c>
       <c r="AD28" t="inlineStr">
@@ -6052,11 +6057,11 @@
         <v>0.014479999</v>
       </c>
       <c r="Y29" t="n">
-        <v>0.76425004</v>
+        <v>0.76403</v>
       </c>
       <c r="AC29" t="inlineStr">
         <is>
-          <t>2026-09-11T22:51:58.984467+00:00</t>
+          <t>2026-09-14T13:18:37.064970+00:00</t>
         </is>
       </c>
       <c r="AD29" t="inlineStr">
@@ -6068,12 +6073,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ServiceNow, Inc.</t>
+          <t>Oracle Corporation</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -6083,72 +6088,69 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Software - Application</t>
+          <t>Software - Infrastructure</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>137017729024</v>
+        <v>432877174784</v>
       </c>
       <c r="F30" t="n">
-        <v>132.5299987792969</v>
+        <v>150.2799987792969</v>
       </c>
       <c r="G30" t="n">
-        <v>14732000256</v>
+        <v>71776002048</v>
       </c>
       <c r="H30" t="n">
-        <v>0.24</v>
+        <v>0.296</v>
       </c>
       <c r="I30" t="n">
-        <v>1.6</v>
+        <v>6.39</v>
       </c>
       <c r="J30" t="n">
-        <v>-0.219</v>
+        <v>0.545</v>
       </c>
       <c r="K30" t="n">
-        <v>5149374976</v>
+        <v>-45853626368</v>
       </c>
       <c r="M30" t="n">
-        <v>4664000000</v>
+        <v>37077000192</v>
       </c>
       <c r="N30" t="n">
-        <v>8453000192</v>
+        <v>169142992896</v>
       </c>
       <c r="O30" t="n">
-        <v>0.74768996</v>
+        <v>0.63957</v>
       </c>
       <c r="P30" t="n">
-        <v>0.04063</v>
+        <v>0.35632</v>
       </c>
       <c r="Q30" t="n">
-        <v>82.831245</v>
+        <v>23.517998</v>
       </c>
       <c r="R30" t="n">
-        <v>9.300687999999999</v>
-      </c>
-      <c r="S30" t="n">
-        <v>26.60861360118592</v>
+        <v>6.030946</v>
       </c>
       <c r="T30" t="n">
-        <v>0.06074912909858599</v>
+        <v>-0.01957202520806123</v>
       </c>
       <c r="U30" t="n">
-        <v>0.2974057444896017</v>
+        <v>-0.1809981083228803</v>
       </c>
       <c r="V30" t="n">
-        <v>0.1664319272627697</v>
+        <v>-0.02437296863035288</v>
       </c>
       <c r="W30" t="n">
-        <v>-0.2937609528009898</v>
+        <v>-0.5062923382987412</v>
       </c>
       <c r="X30" t="n">
-        <v>0.0017499999</v>
+        <v>0.40498</v>
       </c>
       <c r="Y30" t="n">
-        <v>0.84929</v>
+        <v>0.45753</v>
       </c>
       <c r="AC30" t="inlineStr">
         <is>
-          <t>2026-09-11T22:52:07.996492+00:00</t>
+          <t>2026-09-14T13:18:39.625109+00:00</t>
         </is>
       </c>
       <c r="AD30" t="inlineStr">
@@ -6160,12 +6162,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Oracle Corporation</t>
+          <t>ServiceNow, Inc.</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -6175,69 +6177,72 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Software - Infrastructure</t>
+          <t>Software - Application</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>432877174784</v>
+        <v>137017729024</v>
       </c>
       <c r="F31" t="n">
-        <v>150.2799987792969</v>
+        <v>132.5299987792969</v>
       </c>
       <c r="G31" t="n">
-        <v>67356999680</v>
+        <v>14732000256</v>
       </c>
       <c r="H31" t="n">
-        <v>0.206</v>
+        <v>0.24</v>
       </c>
       <c r="I31" t="n">
-        <v>6.38</v>
+        <v>1.6</v>
       </c>
       <c r="J31" t="n">
-        <v>0.219</v>
+        <v>-0.219</v>
       </c>
       <c r="K31" t="n">
-        <v>-24536750080</v>
+        <v>5149374976</v>
       </c>
       <c r="M31" t="n">
-        <v>31893999616</v>
+        <v>4664000000</v>
       </c>
       <c r="N31" t="n">
-        <v>167431995392</v>
+        <v>8453000192</v>
       </c>
       <c r="O31" t="n">
-        <v>0.65822</v>
+        <v>0.74768996</v>
       </c>
       <c r="P31" t="n">
-        <v>0.36202</v>
+        <v>0.04063</v>
       </c>
       <c r="Q31" t="n">
-        <v>23.55486</v>
+        <v>82.831245</v>
       </c>
       <c r="R31" t="n">
-        <v>6.42661</v>
+        <v>9.300687999999999</v>
+      </c>
+      <c r="S31" t="n">
+        <v>26.60861360118592</v>
       </c>
       <c r="T31" t="n">
-        <v>-0.01957202520806123</v>
+        <v>0.06074912909858599</v>
       </c>
       <c r="U31" t="n">
-        <v>-0.1809981083228803</v>
+        <v>0.2974057444896017</v>
       </c>
       <c r="V31" t="n">
-        <v>-0.02437296863035288</v>
+        <v>0.1664319272627697</v>
       </c>
       <c r="W31" t="n">
-        <v>-0.5062922888006263</v>
+        <v>-0.2937609528009898</v>
       </c>
       <c r="X31" t="n">
-        <v>0.40498</v>
+        <v>0.0017499999</v>
       </c>
       <c r="Y31" t="n">
-        <v>0.45806998</v>
+        <v>0.84935</v>
       </c>
       <c r="AC31" t="inlineStr">
         <is>
-          <t>2026-09-11T22:52:01.624013+00:00</t>
+          <t>2026-09-14T13:18:44.780656+00:00</t>
         </is>
       </c>
       <c r="AD31" t="inlineStr">
@@ -6888,7 +6893,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -6922,7 +6927,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -7169,18 +7174,23 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>100</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="C30" t="n">
-        <v>100</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
           <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>price_to_fcf</t>
         </is>
       </c>
       <c r="G30" t="n">
@@ -7198,23 +7208,18 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>94.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="C31" t="n">
-        <v>94.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
           <t>HIGH</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>price_to_fcf</t>
         </is>
       </c>
       <c r="G31" t="n">

</xml_diff>